<commit_message>
final changes to folder structure
</commit_message>
<xml_diff>
--- a/data/raw/Distribution_Connected_Solar_Ge_in_Ireland.xlsx
+++ b/data/raw/Distribution_Connected_Solar_Ge_in_Ireland.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dissertation\Energy\renewcast-ireland\renewcast_ireland\data\raw\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\GitHub\Ireland-energy-forecast\data\raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC846ACA-31FF-4E37-8190-21123C110F5A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD726D80-7EC1-4B0C-8EF9-7C828AFF90DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView minimized="1" xWindow="2652" yWindow="2652" windowWidth="17280" windowHeight="8880" xr2:uid="{894C77AD-9656-43F4-9553-DFC80D80ED54}"/>
+    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="13056" xr2:uid="{894C77AD-9656-43F4-9553-DFC80D80ED54}"/>
   </bookViews>
   <sheets>
     <sheet name="Distribution_Connected_Solar_Ge" sheetId="1" r:id="rId1"/>
@@ -1168,7 +1168,7 @@
     <col min="1" max="1" width="39" customWidth="1"/>
     <col min="2" max="2" width="37.77734375" customWidth="1"/>
     <col min="3" max="3" width="35.21875" customWidth="1"/>
-    <col min="4" max="4" width="9" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="22.44140625" customWidth="1"/>
     <col min="5" max="5" width="14.21875" customWidth="1"/>
     <col min="6" max="6" width="20.33203125" customWidth="1"/>
     <col min="8" max="8" width="8.109375" customWidth="1"/>
@@ -1209,22 +1209,22 @@
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A2" s="5" t="s">
-        <v>10</v>
+        <v>93</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>11</v>
+        <v>94</v>
       </c>
       <c r="C2" s="7" t="s">
         <v>12</v>
       </c>
       <c r="D2" s="8">
-        <v>14</v>
+        <v>0.04</v>
       </c>
       <c r="E2" s="7" t="s">
-        <v>13</v>
+        <v>95</v>
       </c>
       <c r="F2" s="7" t="s">
-        <v>14</v>
+        <v>96</v>
       </c>
       <c r="G2" s="7" t="s">
         <v>15</v>
@@ -1233,30 +1233,30 @@
         <v>16</v>
       </c>
       <c r="I2" s="9">
-        <v>44743</v>
+        <v>41963</v>
       </c>
       <c r="J2" s="10" t="s">
-        <v>17</v>
+        <v>63</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A3" s="11" t="s">
-        <v>18</v>
+        <v>97</v>
       </c>
       <c r="B3" s="12" t="s">
-        <v>19</v>
+        <v>98</v>
       </c>
       <c r="C3" s="13" t="s">
         <v>12</v>
       </c>
       <c r="D3" s="14">
-        <v>10</v>
+        <v>0.02</v>
       </c>
       <c r="E3" s="13" t="s">
-        <v>13</v>
+        <v>99</v>
       </c>
       <c r="F3" s="13" t="s">
-        <v>20</v>
+        <v>100</v>
       </c>
       <c r="G3" s="13" t="s">
         <v>15</v>
@@ -1265,126 +1265,126 @@
         <v>16</v>
       </c>
       <c r="I3" s="15">
-        <v>45058</v>
+        <v>42382</v>
       </c>
       <c r="J3" s="16" t="s">
-        <v>17</v>
+        <v>63</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A4" s="11" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="B4" s="12" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="C4" s="13" t="s">
         <v>12</v>
       </c>
       <c r="D4" s="14">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E4" s="13" t="s">
         <v>13</v>
       </c>
       <c r="F4" s="13" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="G4" s="13" t="s">
-        <v>24</v>
+        <v>15</v>
       </c>
       <c r="H4" s="13" t="s">
         <v>16</v>
       </c>
       <c r="I4" s="15">
-        <v>45276</v>
+        <v>44676</v>
       </c>
       <c r="J4" s="16" t="s">
-        <v>17</v>
+        <v>28</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A5" s="11" t="s">
-        <v>25</v>
+        <v>76</v>
       </c>
       <c r="B5" s="12" t="s">
-        <v>26</v>
+        <v>77</v>
       </c>
       <c r="C5" s="13" t="s">
         <v>12</v>
       </c>
       <c r="D5" s="14">
-        <v>8</v>
+        <v>0.12</v>
       </c>
       <c r="E5" s="13" t="s">
-        <v>13</v>
+        <v>78</v>
       </c>
       <c r="F5" s="13" t="s">
-        <v>27</v>
+        <v>79</v>
       </c>
       <c r="G5" s="13" t="s">
-        <v>15</v>
+        <v>71</v>
       </c>
       <c r="H5" s="13" t="s">
         <v>16</v>
       </c>
       <c r="I5" s="15">
-        <v>44676</v>
+        <v>44692</v>
       </c>
       <c r="J5" s="16" t="s">
-        <v>28</v>
+        <v>63</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A6" s="11" t="s">
-        <v>29</v>
+        <v>80</v>
       </c>
       <c r="B6" s="12" t="s">
-        <v>30</v>
+        <v>81</v>
       </c>
       <c r="C6" s="13" t="s">
         <v>12</v>
       </c>
       <c r="D6" s="14">
-        <v>7.98</v>
+        <v>0.1</v>
       </c>
       <c r="E6" s="13" t="s">
-        <v>31</v>
+        <v>82</v>
       </c>
       <c r="F6" s="13" t="s">
-        <v>32</v>
+        <v>83</v>
       </c>
       <c r="G6" s="13" t="s">
-        <v>15</v>
+        <v>71</v>
       </c>
       <c r="H6" s="13" t="s">
         <v>16</v>
       </c>
       <c r="I6" s="15">
-        <v>44793</v>
+        <v>44692</v>
       </c>
       <c r="J6" s="16" t="s">
-        <v>17</v>
+        <v>63</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A7" s="11" t="s">
-        <v>33</v>
+        <v>10</v>
       </c>
       <c r="B7" s="12" t="s">
-        <v>34</v>
+        <v>11</v>
       </c>
       <c r="C7" s="13" t="s">
         <v>12</v>
       </c>
       <c r="D7" s="14">
-        <v>4.99</v>
+        <v>14</v>
       </c>
       <c r="E7" s="13" t="s">
-        <v>35</v>
+        <v>13</v>
       </c>
       <c r="F7" s="13" t="s">
-        <v>36</v>
+        <v>14</v>
       </c>
       <c r="G7" s="13" t="s">
         <v>15</v>
@@ -1393,7 +1393,7 @@
         <v>16</v>
       </c>
       <c r="I7" s="15">
-        <v>44839</v>
+        <v>44743</v>
       </c>
       <c r="J7" s="16" t="s">
         <v>17</v>
@@ -1401,22 +1401,22 @@
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A8" s="11" t="s">
-        <v>37</v>
+        <v>51</v>
       </c>
       <c r="B8" s="12" t="s">
-        <v>38</v>
+        <v>52</v>
       </c>
       <c r="C8" s="13" t="s">
         <v>12</v>
       </c>
       <c r="D8" s="14">
-        <v>4.95</v>
+        <v>3.99</v>
       </c>
       <c r="E8" s="13" t="s">
-        <v>39</v>
+        <v>53</v>
       </c>
       <c r="F8" s="13" t="s">
-        <v>40</v>
+        <v>54</v>
       </c>
       <c r="G8" s="13" t="s">
         <v>15</v>
@@ -1425,71 +1425,71 @@
         <v>16</v>
       </c>
       <c r="I8" s="15">
-        <v>45344</v>
+        <v>44768</v>
       </c>
       <c r="J8" s="16" t="s">
-        <v>17</v>
+        <v>28</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A9" s="11" t="s">
-        <v>41</v>
+        <v>29</v>
       </c>
       <c r="B9" s="12" t="s">
-        <v>42</v>
+        <v>30</v>
       </c>
       <c r="C9" s="13" t="s">
         <v>12</v>
       </c>
       <c r="D9" s="14">
-        <v>4.95</v>
+        <v>7.98</v>
       </c>
       <c r="E9" s="13" t="s">
-        <v>43</v>
+        <v>31</v>
       </c>
       <c r="F9" s="13" t="s">
         <v>32</v>
       </c>
       <c r="G9" s="13" t="s">
-        <v>24</v>
+        <v>15</v>
       </c>
       <c r="H9" s="13" t="s">
         <v>16</v>
       </c>
       <c r="I9" s="15">
-        <v>44872</v>
+        <v>44793</v>
       </c>
       <c r="J9" s="16" t="s">
-        <v>44</v>
+        <v>17</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A10" s="11" t="s">
-        <v>45</v>
+        <v>33</v>
       </c>
       <c r="B10" s="12" t="s">
-        <v>46</v>
+        <v>34</v>
       </c>
       <c r="C10" s="13" t="s">
         <v>12</v>
       </c>
       <c r="D10" s="14">
-        <v>4</v>
+        <v>4.99</v>
       </c>
       <c r="E10" s="13" t="s">
-        <v>13</v>
+        <v>35</v>
       </c>
       <c r="F10" s="13" t="s">
-        <v>47</v>
+        <v>36</v>
       </c>
       <c r="G10" s="13" t="s">
-        <v>24</v>
+        <v>15</v>
       </c>
       <c r="H10" s="13" t="s">
         <v>16</v>
       </c>
       <c r="I10" s="15">
-        <v>45175</v>
+        <v>44839</v>
       </c>
       <c r="J10" s="16" t="s">
         <v>17</v>
@@ -1497,31 +1497,31 @@
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A11" s="11" t="s">
-        <v>48</v>
+        <v>41</v>
       </c>
       <c r="B11" s="12" t="s">
-        <v>49</v>
+        <v>42</v>
       </c>
       <c r="C11" s="13" t="s">
         <v>12</v>
       </c>
       <c r="D11" s="14">
-        <v>4</v>
+        <v>4.95</v>
       </c>
       <c r="E11" s="13" t="s">
-        <v>13</v>
+        <v>43</v>
       </c>
       <c r="F11" s="13" t="s">
-        <v>50</v>
+        <v>32</v>
       </c>
       <c r="G11" s="13" t="s">
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="H11" s="13" t="s">
         <v>16</v>
       </c>
       <c r="I11" s="15">
-        <v>44917</v>
+        <v>44872</v>
       </c>
       <c r="J11" s="16" t="s">
         <v>44</v>
@@ -1529,31 +1529,31 @@
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A12" s="11" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="B12" s="12" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="C12" s="13" t="s">
         <v>12</v>
       </c>
       <c r="D12" s="14">
-        <v>3.99</v>
+        <v>3.6</v>
       </c>
       <c r="E12" s="13" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="F12" s="13" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="G12" s="13" t="s">
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="H12" s="13" t="s">
         <v>16</v>
       </c>
       <c r="I12" s="15">
-        <v>44768</v>
+        <v>44909</v>
       </c>
       <c r="J12" s="16" t="s">
         <v>28</v>
@@ -1561,63 +1561,63 @@
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A13" s="11" t="s">
-        <v>55</v>
+        <v>48</v>
       </c>
       <c r="B13" s="12" t="s">
-        <v>56</v>
+        <v>49</v>
       </c>
       <c r="C13" s="13" t="s">
         <v>12</v>
       </c>
       <c r="D13" s="14">
-        <v>3.6</v>
+        <v>4</v>
       </c>
       <c r="E13" s="13" t="s">
-        <v>57</v>
+        <v>13</v>
       </c>
       <c r="F13" s="13" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="G13" s="13" t="s">
-        <v>24</v>
+        <v>15</v>
       </c>
       <c r="H13" s="13" t="s">
         <v>16</v>
       </c>
       <c r="I13" s="15">
-        <v>44909</v>
+        <v>44917</v>
       </c>
       <c r="J13" s="16" t="s">
-        <v>28</v>
+        <v>44</v>
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A14" s="11" t="s">
-        <v>59</v>
+        <v>67</v>
       </c>
       <c r="B14" s="12" t="s">
-        <v>60</v>
+        <v>68</v>
       </c>
       <c r="C14" s="13" t="s">
         <v>12</v>
       </c>
       <c r="D14" s="14">
-        <v>0.499</v>
+        <v>0.3</v>
       </c>
       <c r="E14" s="13" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="F14" s="13" t="s">
-        <v>62</v>
+        <v>70</v>
       </c>
       <c r="G14" s="13" t="s">
-        <v>15</v>
+        <v>71</v>
       </c>
       <c r="H14" s="13" t="s">
         <v>16</v>
       </c>
       <c r="I14" s="15">
-        <v>45177</v>
+        <v>45015</v>
       </c>
       <c r="J14" s="16" t="s">
         <v>63</v>
@@ -1625,54 +1625,54 @@
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A15" s="11" t="s">
-        <v>64</v>
+        <v>72</v>
       </c>
       <c r="B15" s="12" t="s">
-        <v>65</v>
+        <v>73</v>
       </c>
       <c r="C15" s="13" t="s">
         <v>12</v>
       </c>
       <c r="D15" s="14">
-        <v>0.34</v>
+        <v>0.18</v>
       </c>
       <c r="E15" s="13" t="s">
-        <v>57</v>
+        <v>74</v>
       </c>
       <c r="F15" s="13" t="s">
-        <v>58</v>
+        <v>75</v>
       </c>
       <c r="G15" s="13" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="H15" s="13" t="s">
         <v>16</v>
       </c>
       <c r="I15" s="15">
-        <v>45108</v>
+        <v>45020</v>
       </c>
       <c r="J15" s="16" t="s">
-        <v>28</v>
+        <v>63</v>
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A16" s="11" t="s">
-        <v>67</v>
+        <v>84</v>
       </c>
       <c r="B16" s="12" t="s">
-        <v>68</v>
+        <v>85</v>
       </c>
       <c r="C16" s="13" t="s">
         <v>12</v>
       </c>
       <c r="D16" s="14">
-        <v>0.3</v>
+        <v>7.0000000000000007E-2</v>
       </c>
       <c r="E16" s="13" t="s">
-        <v>69</v>
+        <v>86</v>
       </c>
       <c r="F16" s="13" t="s">
-        <v>70</v>
+        <v>87</v>
       </c>
       <c r="G16" s="13" t="s">
         <v>71</v>
@@ -1681,7 +1681,7 @@
         <v>16</v>
       </c>
       <c r="I16" s="15">
-        <v>45015</v>
+        <v>45041</v>
       </c>
       <c r="J16" s="16" t="s">
         <v>63</v>
@@ -1689,127 +1689,127 @@
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A17" s="11" t="s">
-        <v>72</v>
+        <v>18</v>
       </c>
       <c r="B17" s="12" t="s">
-        <v>73</v>
+        <v>19</v>
       </c>
       <c r="C17" s="13" t="s">
         <v>12</v>
       </c>
       <c r="D17" s="14">
-        <v>0.18</v>
+        <v>10</v>
       </c>
       <c r="E17" s="13" t="s">
-        <v>74</v>
+        <v>13</v>
       </c>
       <c r="F17" s="13" t="s">
-        <v>75</v>
+        <v>20</v>
       </c>
       <c r="G17" s="13" t="s">
-        <v>71</v>
+        <v>15</v>
       </c>
       <c r="H17" s="13" t="s">
         <v>16</v>
       </c>
       <c r="I17" s="15">
-        <v>45020</v>
+        <v>45058</v>
       </c>
       <c r="J17" s="16" t="s">
-        <v>63</v>
+        <v>17</v>
       </c>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A18" s="11" t="s">
-        <v>76</v>
+        <v>64</v>
       </c>
       <c r="B18" s="12" t="s">
-        <v>77</v>
+        <v>65</v>
       </c>
       <c r="C18" s="13" t="s">
         <v>12</v>
       </c>
       <c r="D18" s="14">
-        <v>0.12</v>
+        <v>0.34</v>
       </c>
       <c r="E18" s="13" t="s">
-        <v>78</v>
+        <v>57</v>
       </c>
       <c r="F18" s="13" t="s">
-        <v>79</v>
+        <v>58</v>
       </c>
       <c r="G18" s="13" t="s">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="H18" s="13" t="s">
         <v>16</v>
       </c>
       <c r="I18" s="15">
-        <v>44692</v>
+        <v>45108</v>
       </c>
       <c r="J18" s="16" t="s">
-        <v>63</v>
+        <v>28</v>
       </c>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A19" s="11" t="s">
-        <v>80</v>
+        <v>45</v>
       </c>
       <c r="B19" s="12" t="s">
-        <v>81</v>
+        <v>46</v>
       </c>
       <c r="C19" s="13" t="s">
         <v>12</v>
       </c>
       <c r="D19" s="14">
-        <v>0.1</v>
+        <v>4</v>
       </c>
       <c r="E19" s="13" t="s">
-        <v>82</v>
+        <v>13</v>
       </c>
       <c r="F19" s="13" t="s">
-        <v>83</v>
+        <v>47</v>
       </c>
       <c r="G19" s="13" t="s">
-        <v>71</v>
+        <v>24</v>
       </c>
       <c r="H19" s="13" t="s">
         <v>16</v>
       </c>
       <c r="I19" s="15">
-        <v>44692</v>
+        <v>45175</v>
       </c>
       <c r="J19" s="16" t="s">
-        <v>63</v>
+        <v>17</v>
       </c>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A20" s="11" t="s">
-        <v>84</v>
+        <v>59</v>
       </c>
       <c r="B20" s="12" t="s">
-        <v>85</v>
+        <v>60</v>
       </c>
       <c r="C20" s="13" t="s">
         <v>12</v>
       </c>
       <c r="D20" s="14">
-        <v>7.0000000000000007E-2</v>
+        <v>0.499</v>
       </c>
       <c r="E20" s="13" t="s">
-        <v>86</v>
+        <v>61</v>
       </c>
       <c r="F20" s="13" t="s">
-        <v>87</v>
+        <v>62</v>
       </c>
       <c r="G20" s="13" t="s">
-        <v>71</v>
+        <v>15</v>
       </c>
       <c r="H20" s="13" t="s">
         <v>16</v>
       </c>
       <c r="I20" s="15">
-        <v>45041</v>
+        <v>45177</v>
       </c>
       <c r="J20" s="16" t="s">
         <v>63</v>
@@ -1817,54 +1817,54 @@
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A21" s="11" t="s">
-        <v>88</v>
+        <v>21</v>
       </c>
       <c r="B21" s="12" t="s">
-        <v>89</v>
+        <v>22</v>
       </c>
       <c r="C21" s="13" t="s">
         <v>12</v>
       </c>
       <c r="D21" s="14">
-        <v>0.05</v>
+        <v>9</v>
       </c>
       <c r="E21" s="13" t="s">
         <v>13</v>
       </c>
       <c r="F21" s="13" t="s">
-        <v>90</v>
+        <v>23</v>
       </c>
       <c r="G21" s="13" t="s">
-        <v>91</v>
+        <v>24</v>
       </c>
       <c r="H21" s="13" t="s">
         <v>16</v>
       </c>
-      <c r="I21" s="15" t="s">
-        <v>92</v>
+      <c r="I21" s="15">
+        <v>45276</v>
       </c>
       <c r="J21" s="16" t="s">
-        <v>28</v>
+        <v>17</v>
       </c>
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A22" s="11" t="s">
-        <v>93</v>
+        <v>37</v>
       </c>
       <c r="B22" s="12" t="s">
-        <v>94</v>
+        <v>38</v>
       </c>
       <c r="C22" s="13" t="s">
         <v>12</v>
       </c>
       <c r="D22" s="14">
-        <v>0.04</v>
+        <v>4.95</v>
       </c>
       <c r="E22" s="13" t="s">
-        <v>95</v>
+        <v>39</v>
       </c>
       <c r="F22" s="13" t="s">
-        <v>96</v>
+        <v>40</v>
       </c>
       <c r="G22" s="13" t="s">
         <v>15</v>
@@ -1873,30 +1873,30 @@
         <v>16</v>
       </c>
       <c r="I22" s="15">
-        <v>41963</v>
+        <v>45344</v>
       </c>
       <c r="J22" s="16" t="s">
-        <v>63</v>
+        <v>17</v>
       </c>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A23" s="11" t="s">
-        <v>97</v>
+        <v>140</v>
       </c>
       <c r="B23" s="12" t="s">
-        <v>98</v>
+        <v>141</v>
       </c>
       <c r="C23" s="13" t="s">
         <v>12</v>
       </c>
       <c r="D23" s="14">
-        <v>0.02</v>
+        <v>3.99</v>
       </c>
       <c r="E23" s="13" t="s">
-        <v>99</v>
+        <v>142</v>
       </c>
       <c r="F23" s="13" t="s">
-        <v>100</v>
+        <v>143</v>
       </c>
       <c r="G23" s="13" t="s">
         <v>15</v>
@@ -1905,7 +1905,7 @@
         <v>16</v>
       </c>
       <c r="I23" s="15">
-        <v>42382</v>
+        <v>45392</v>
       </c>
       <c r="J23" s="16" t="s">
         <v>63</v>
@@ -1913,22 +1913,22 @@
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A24" s="11" t="s">
-        <v>101</v>
+        <v>109</v>
       </c>
       <c r="B24" s="12" t="s">
-        <v>102</v>
+        <v>110</v>
       </c>
       <c r="C24" s="13" t="s">
         <v>12</v>
       </c>
       <c r="D24" s="14">
-        <v>0.19</v>
+        <v>0.12</v>
       </c>
       <c r="E24" s="13" t="s">
-        <v>103</v>
+        <v>111</v>
       </c>
       <c r="F24" s="13" t="s">
-        <v>104</v>
+        <v>112</v>
       </c>
       <c r="G24" s="13" t="s">
         <v>66</v>
@@ -1937,7 +1937,7 @@
         <v>16</v>
       </c>
       <c r="I24" s="15">
-        <v>45455</v>
+        <v>45400</v>
       </c>
       <c r="J24" s="16" t="s">
         <v>63</v>
@@ -1945,22 +1945,22 @@
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A25" s="11" t="s">
-        <v>105</v>
+        <v>124</v>
       </c>
       <c r="B25" s="12" t="s">
-        <v>106</v>
+        <v>125</v>
       </c>
       <c r="C25" s="13" t="s">
         <v>12</v>
       </c>
       <c r="D25" s="14">
-        <v>4</v>
+        <v>7.14</v>
       </c>
       <c r="E25" s="13" t="s">
-        <v>107</v>
+        <v>126</v>
       </c>
       <c r="F25" s="13" t="s">
-        <v>108</v>
+        <v>127</v>
       </c>
       <c r="G25" s="13" t="s">
         <v>15</v>
@@ -1969,50 +1969,50 @@
         <v>16</v>
       </c>
       <c r="I25" s="15">
-        <v>45469</v>
+        <v>45413</v>
       </c>
       <c r="J25" s="16" t="s">
-        <v>28</v>
+        <v>17</v>
       </c>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A26" s="11" t="s">
-        <v>109</v>
+        <v>121</v>
       </c>
       <c r="B26" s="12" t="s">
-        <v>110</v>
+        <v>122</v>
       </c>
       <c r="C26" s="13" t="s">
         <v>12</v>
       </c>
       <c r="D26" s="14">
-        <v>0.12</v>
+        <v>4.95</v>
       </c>
       <c r="E26" s="13" t="s">
-        <v>111</v>
+        <v>123</v>
       </c>
       <c r="F26" s="13" t="s">
-        <v>112</v>
+        <v>40</v>
       </c>
       <c r="G26" s="13" t="s">
-        <v>66</v>
+        <v>15</v>
       </c>
       <c r="H26" s="13" t="s">
         <v>16</v>
       </c>
       <c r="I26" s="15">
-        <v>45400</v>
+        <v>45415</v>
       </c>
       <c r="J26" s="16" t="s">
-        <v>63</v>
+        <v>17</v>
       </c>
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A27" s="11" t="s">
-        <v>113</v>
+        <v>117</v>
       </c>
       <c r="B27" s="12" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="C27" s="13" t="s">
         <v>12</v>
@@ -2021,10 +2021,10 @@
         <v>4.95</v>
       </c>
       <c r="E27" s="13" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="F27" s="13" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="G27" s="13" t="s">
         <v>15</v>
@@ -2033,7 +2033,7 @@
         <v>16</v>
       </c>
       <c r="I27" s="15">
-        <v>45429</v>
+        <v>45421</v>
       </c>
       <c r="J27" s="16" t="s">
         <v>28</v>
@@ -2041,10 +2041,10 @@
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A28" s="11" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="B28" s="12" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="C28" s="13" t="s">
         <v>12</v>
@@ -2053,10 +2053,10 @@
         <v>4.95</v>
       </c>
       <c r="E28" s="13" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="F28" s="13" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="G28" s="13" t="s">
         <v>15</v>
@@ -2065,7 +2065,7 @@
         <v>16</v>
       </c>
       <c r="I28" s="15">
-        <v>45421</v>
+        <v>45429</v>
       </c>
       <c r="J28" s="16" t="s">
         <v>28</v>
@@ -2073,54 +2073,54 @@
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A29" s="11" t="s">
-        <v>121</v>
+        <v>101</v>
       </c>
       <c r="B29" s="12" t="s">
-        <v>122</v>
+        <v>102</v>
       </c>
       <c r="C29" s="13" t="s">
         <v>12</v>
       </c>
       <c r="D29" s="14">
-        <v>4.95</v>
+        <v>0.19</v>
       </c>
       <c r="E29" s="13" t="s">
-        <v>123</v>
+        <v>103</v>
       </c>
       <c r="F29" s="13" t="s">
-        <v>40</v>
+        <v>104</v>
       </c>
       <c r="G29" s="13" t="s">
-        <v>15</v>
+        <v>66</v>
       </c>
       <c r="H29" s="13" t="s">
         <v>16</v>
       </c>
       <c r="I29" s="15">
-        <v>45415</v>
+        <v>45455</v>
       </c>
       <c r="J29" s="16" t="s">
-        <v>17</v>
+        <v>63</v>
       </c>
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A30" s="11" t="s">
-        <v>124</v>
+        <v>105</v>
       </c>
       <c r="B30" s="12" t="s">
-        <v>125</v>
+        <v>106</v>
       </c>
       <c r="C30" s="13" t="s">
         <v>12</v>
       </c>
       <c r="D30" s="14">
-        <v>7.14</v>
+        <v>4</v>
       </c>
       <c r="E30" s="13" t="s">
-        <v>126</v>
+        <v>107</v>
       </c>
       <c r="F30" s="13" t="s">
-        <v>127</v>
+        <v>108</v>
       </c>
       <c r="G30" s="13" t="s">
         <v>15</v>
@@ -2129,39 +2129,39 @@
         <v>16</v>
       </c>
       <c r="I30" s="15">
-        <v>45413</v>
+        <v>45469</v>
       </c>
       <c r="J30" s="16" t="s">
-        <v>17</v>
+        <v>28</v>
       </c>
     </row>
     <row r="31" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A31" s="11" t="s">
-        <v>128</v>
+        <v>136</v>
       </c>
       <c r="B31" s="12" t="s">
-        <v>129</v>
+        <v>137</v>
       </c>
       <c r="C31" s="13" t="s">
         <v>12</v>
       </c>
       <c r="D31" s="14">
-        <v>0.2</v>
+        <v>4.95</v>
       </c>
       <c r="E31" s="13" t="s">
-        <v>126</v>
+        <v>138</v>
       </c>
       <c r="F31" s="13" t="s">
-        <v>130</v>
+        <v>139</v>
       </c>
       <c r="G31" s="13" t="s">
-        <v>131</v>
+        <v>15</v>
       </c>
       <c r="H31" s="13" t="s">
         <v>16</v>
       </c>
       <c r="I31" s="15">
-        <v>45559</v>
+        <v>45498</v>
       </c>
       <c r="J31" s="16" t="s">
         <v>28</v>
@@ -2201,31 +2201,31 @@
     </row>
     <row r="33" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A33" s="11" t="s">
-        <v>136</v>
+        <v>128</v>
       </c>
       <c r="B33" s="12" t="s">
-        <v>137</v>
+        <v>129</v>
       </c>
       <c r="C33" s="13" t="s">
         <v>12</v>
       </c>
       <c r="D33" s="14">
-        <v>4.95</v>
+        <v>0.2</v>
       </c>
       <c r="E33" s="13" t="s">
-        <v>138</v>
+        <v>126</v>
       </c>
       <c r="F33" s="13" t="s">
-        <v>139</v>
+        <v>130</v>
       </c>
       <c r="G33" s="13" t="s">
-        <v>15</v>
+        <v>131</v>
       </c>
       <c r="H33" s="13" t="s">
         <v>16</v>
       </c>
       <c r="I33" s="15">
-        <v>45498</v>
+        <v>45559</v>
       </c>
       <c r="J33" s="16" t="s">
         <v>28</v>
@@ -2233,66 +2233,66 @@
     </row>
     <row r="34" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A34" s="11" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
       <c r="B34" s="12" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
       <c r="C34" s="13" t="s">
         <v>12</v>
       </c>
       <c r="D34" s="14">
-        <v>3.99</v>
+        <v>21</v>
       </c>
       <c r="E34" s="13" t="s">
-        <v>142</v>
+        <v>126</v>
       </c>
       <c r="F34" s="13" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="G34" s="13" t="s">
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="H34" s="13" t="s">
         <v>16</v>
       </c>
       <c r="I34" s="15">
-        <v>45392</v>
+        <v>45579</v>
       </c>
       <c r="J34" s="16" t="s">
-        <v>63</v>
+        <v>44</v>
       </c>
     </row>
     <row r="35" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A35" s="11" t="s">
-        <v>144</v>
+        <v>151</v>
       </c>
       <c r="B35" s="12" t="s">
-        <v>145</v>
+        <v>152</v>
       </c>
       <c r="C35" s="13" t="s">
         <v>12</v>
       </c>
       <c r="D35" s="14">
-        <v>21</v>
+        <v>4</v>
       </c>
       <c r="E35" s="13" t="s">
         <v>126</v>
       </c>
       <c r="F35" s="13" t="s">
-        <v>146</v>
+        <v>153</v>
       </c>
       <c r="G35" s="13" t="s">
-        <v>24</v>
+        <v>15</v>
       </c>
       <c r="H35" s="13" t="s">
         <v>16</v>
       </c>
       <c r="I35" s="15">
-        <v>45579</v>
+        <v>45615</v>
       </c>
       <c r="J35" s="16" t="s">
-        <v>44</v>
+        <v>17</v>
       </c>
     </row>
     <row r="36" spans="1:10" x14ac:dyDescent="0.3">
@@ -2329,34 +2329,34 @@
     </row>
     <row r="37" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A37" s="17" t="s">
-        <v>151</v>
+        <v>88</v>
       </c>
       <c r="B37" s="18" t="s">
-        <v>152</v>
+        <v>89</v>
       </c>
       <c r="C37" s="19" t="s">
         <v>12</v>
       </c>
       <c r="D37" s="20">
-        <v>4</v>
+        <v>0.05</v>
       </c>
       <c r="E37" s="19" t="s">
-        <v>126</v>
+        <v>13</v>
       </c>
       <c r="F37" s="19" t="s">
-        <v>153</v>
+        <v>90</v>
       </c>
       <c r="G37" s="19" t="s">
-        <v>15</v>
+        <v>91</v>
       </c>
       <c r="H37" s="19" t="s">
         <v>16</v>
       </c>
-      <c r="I37" s="21">
-        <v>45615</v>
+      <c r="I37" s="21" t="s">
+        <v>92</v>
       </c>
       <c r="J37" s="22" t="s">
-        <v>17</v>
+        <v>28</v>
       </c>
     </row>
     <row r="38" spans="1:10" x14ac:dyDescent="0.3">
@@ -2365,7 +2365,7 @@
       </c>
       <c r="D38" s="24">
         <f>SUM(D2:D37)</f>
-        <v>145.91899999999998</v>
+        <v>145.91900000000004</v>
       </c>
     </row>
     <row r="39" spans="1:10" x14ac:dyDescent="0.3">
@@ -2374,6 +2374,9 @@
       </c>
     </row>
   </sheetData>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:J39">
+    <sortCondition ref="I2:I39"/>
+  </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>